<commit_message>
Add missing walmart keyword result
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FHMLu692q2iDkhZE8o5ZpS
</commit_message>
<xml_diff>
--- a/research/niche-keyword-validation.xlsx
+++ b/research/niche-keyword-validation.xlsx
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1034" uniqueCount="245">
   <si>
     <t xml:space="preserve">Niche Keyword Validation – Semrush Check</t>
   </si>
@@ -5326,19 +5326,27 @@
       <c r="E114" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="F114" s="10"/>
-      <c r="G114" s="11"/>
-      <c r="H114" s="12"/>
+      <c r="F114" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G114" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" s="12" t="n">
+        <v>52</v>
+      </c>
       <c r="I114" s="13"/>
-      <c r="J114" s="14" t="str">
+      <c r="J114" s="14" t="n">
         <f aca="false">IF(AND(ISNUMBER(F114),ISNUMBER(G114)),F114*G114,"")</f>
-        <v/>
+        <v>0</v>
       </c>
       <c r="K114" s="9" t="str">
         <f aca="false">IF(H114="","",IF(H114&lt;30,"Easy",IF(H114&lt;50,"Medium",IF(H114&lt;70,"Hard","Very hard"))))</f>
-        <v/>
-      </c>
-      <c r="L114" s="9"/>
+        <v>Hard</v>
+      </c>
+      <c r="L114" s="9" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="9" t="n">
@@ -7644,7 +7652,7 @@
       </c>
       <c r="C7" s="18" t="n">
         <f aca="false">COUNTIFS(Keywords!$B$2:$B$176,A7,Keywords!$F$2:$F$176,"&lt;&gt;")</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D7" s="19" t="n">
         <f aca="false">IF(C7=0,"",SUMIFS(Keywords!$F$2:$F$176,Keywords!$B$2:$B$176,A7))</f>
@@ -7664,11 +7672,11 @@
       </c>
       <c r="H7" s="18" t="n">
         <f aca="false">IFERROR(AVERAGEIFS(Keywords!$H$2:$H$176,Keywords!$B$2:$B$176,A7,Keywords!$H$2:$H$176,"&lt;&gt;"),"")</f>
-        <v>33.5263157894737</v>
+        <v>34.45</v>
       </c>
       <c r="I7" s="18" t="n">
         <f aca="false">IFERROR(AVERAGEIFS(Keywords!$H$2:$H$176,Keywords!$B$2:$B$176,A7,Keywords!$C$2:$C$176,"Agency-side",Keywords!$H$2:$H$176,"&lt;&gt;"),"")</f>
-        <v>33.5263157894737</v>
+        <v>34.45</v>
       </c>
       <c r="J7" s="14" t="n">
         <f aca="false">IF(C7=0,"",SUMIFS(Keywords!$J$2:$J$176,Keywords!$B$2:$B$176,A7))</f>
@@ -7676,7 +7684,7 @@
       </c>
       <c r="K7" s="21" t="n">
         <f aca="false">IF(OR(J7="",H7=""),"",J7/MAX(H7,1))</f>
-        <v>77.6464678178964</v>
+        <v>75.5645863570392</v>
       </c>
       <c r="L7" s="18" t="n">
         <f aca="false">IF(K7="","",COUNTIF($K$5:$K$8,"&gt;"&amp;K7)+1)</f>

</xml_diff>